<commit_message>
docs(assets): regenerate all 12 assets with BeyondNet dark/gold identity and conceptual diagrams
</commit_message>
<xml_diff>
--- a/reference/governance/sdlc/assets/Evolith_Master_Workbook.xlsx
+++ b/reference/governance/sdlc/assets/Evolith_Master_Workbook.xlsx
@@ -9,8 +9,6 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Portada" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_Proyecto" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stakeholders" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan_Fases" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,8 +27,11 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
       <b val="1"/>
-      <color rgb="001E3A5F"/>
+      <color rgb="00CAC5B2"/>
       <sz val="16"/>
     </font>
     <font>
@@ -47,20 +48,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E3A5F"/>
-        <bgColor rgb="001E3A5F"/>
+        <fgColor rgb="00121212"/>
+        <bgColor rgb="00121212"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F3F4F6"/>
-        <bgColor rgb="00F3F4F6"/>
+        <fgColor rgb="002A2A2A"/>
+        <bgColor rgb="002A2A2A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
+        <fgColor rgb="001A1A1A"/>
+        <bgColor rgb="001A1A1A"/>
       </patternFill>
     </fill>
   </fills>
@@ -73,25 +74,34 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="00CAC5B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CAC5B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CAC5B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CAC5B2"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -456,10 +466,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00CAC5B2"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,27 +479,85 @@
           <t>EVOLITH SDLC - Workbook Maestro Integrador</t>
         </is>
       </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Versión 1.0</t>
         </is>
       </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Nivel de Confidencialidad: Uso Interno</t>
         </is>
       </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Instrucciones: Llenar cada pestaña conforme se avanza en la fase correspondiente. Para ser auditado en los Quality Gates.</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Instrucciones: Llenar cada pestaña conforme se avanza en la fase correspondiente.</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -513,380 +582,130 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>ID_Indicador</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Nombre Métrica</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Valor Actual</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Objetivo</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Tendencia</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>IND-01</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Cumplimiento Cronograma</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>&gt; 90%</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Verde</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Estable</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>IND-02</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Cobertura de Pruebas</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>82%</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>&gt; 80%</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Verde</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Al alza</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>IND-03</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Defectos Abiertos Severidad 1</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Rojo</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Estable</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Nombre Completo</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Rol Evolith</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Nivel de Autoridad</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Fases Clave</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Email Corporativo</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Laura Mendes</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Sponsor</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Aprobador (Go/No-Go)</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>F1, F6</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>lmendes@empresa.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Carlos Ruiz</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Dueño Negocio</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>F1, F2, F5</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>cruiz@empresa.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Elena Torres</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Arquitecto Solución</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Dueño Técnico</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>F3, F4</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>etorres@empresa.com</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Fase SDLC</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Hito Principal</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Fecha Planificada</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Fecha Real</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>F1_Ideacion</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Firma Business Case</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Completado</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>F2_Analisis</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Cierre de PRD</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr"/>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>En Progreso</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>F3_Diseno</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Aprobación Blueprint</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
         </is>
       </c>
     </row>

</xml_diff>